<commit_message>
ovl/zpra_dpr: 27.10.2026 workbook - actions addressed to the data source
M	ovl/zpra_dpr/reconciliation/2026-10-27/DPR_QAS_vs_PRD_27.10.2026.xlsx
M	ovl/zpra_dpr/reconciliation/2026-10-27/README.md

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ovl/zpra_dpr/reconciliation/2026-10-27/DPR_QAS_vs_PRD_27.10.2026.xlsx
+++ b/ovl/zpra_dpr/reconciliation/2026-10-27/DPR_QAS_vs_PRD_27.10.2026.xlsx
@@ -519,7 +519,7 @@
     <row r="5" ht="48" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Oil (NET_PROD) is mostly correct. Gas is wrong for RUS_SK1 (unit problem), BRA_BC1 and COL_CPO. Some values never arrive. Comments are wrong. All causes are in the CPI mapping / source report, not in the ABAP class.</t>
+          <t>Oil (NET_PROD) is mostly correct. Gas is wrong for RUS_SK1 (unit problem), BRA_BC1 and COL_CPO. Some values never arrive. Comments are wrong. The interface passes values as received, so the differences come from the source file.</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>RUS_SK1 gas is 28.3168 times too small in Quality on every gas row (13 rows). Example: ARKUTUN gross gas Production 2,973,887 vs Quality 105,022. Quality holds MCF (thousand cubic feet) but the system labels it M3.</t>
+          <t>RUS_SK1 gas is 28.3168 times too small in Quality on every gas row (13 rows). Example: ARKUTUN gross gas Production 2,973,887 vs Quality 105,022. The value in the file is MCF (thousand cubic feet) but is labelled M3.</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>CPI: convert MCF to m3 (multiply by 28.3168) before posting.</t>
+          <t>Source: send gas in m3 (multiply MCF by 28.3168).</t>
         </is>
       </c>
     </row>
@@ -625,7 +625,7 @@
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>CPI: check which source column is mapped.</t>
+          <t>Source: check which column is used for this measure.</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>CPI: divide by 1,000,000 (m3 to MCM).</t>
+          <t>Source: send MCM (divide m3 by 1,000,000).</t>
         </is>
       </c>
     </row>
@@ -665,7 +665,7 @@
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>Confirm with Colombia asset which figure is final; re-run if source changed.</t>
+          <t>Source: confirm the final figure with the Colombia asset and resend.</t>
         </is>
       </c>
     </row>
@@ -685,7 +685,7 @@
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>CPI: map these measures; check the payload.</t>
+          <t>Source: include these measures in the file.</t>
         </is>
       </c>
     </row>
@@ -705,7 +705,7 @@
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>CPI: add block value mapping.</t>
+          <t>Source: send the block codes SAP uses.</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
-          <t>CPI: map the remark column, not neighbouring cells.</t>
+          <t>Source: put the remark in the comment field only.</t>
         </is>
       </c>
     </row>
@@ -745,7 +745,7 @@
       </c>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>Information only - agree with DPR team if zero rows are needed.</t>
+          <t>Information only - not an error; agree with DPR team if zero rows are needed.</t>
         </is>
       </c>
     </row>
@@ -9757,7 +9757,7 @@
       </c>
       <c r="K2" s="9" t="inlineStr">
         <is>
-          <t>Convert m3 to MCM in CPI.</t>
+          <t>Source to send gas in MCM (file holds m3).</t>
         </is>
       </c>
     </row>
@@ -9808,7 +9808,7 @@
       </c>
       <c r="K3" s="9" t="inlineStr">
         <is>
-          <t>Confirm against source report; QAS run may predate asset correction.</t>
+          <t>Source to confirm the final figure; the Quality run may predate the asset correction.</t>
         </is>
       </c>
     </row>
@@ -9857,7 +9857,7 @@
       </c>
       <c r="K4" s="9" t="inlineStr">
         <is>
-          <t>Check CPI payload / mapping for this measure.</t>
+          <t>Source to include this measure in the file.</t>
         </is>
       </c>
     </row>
@@ -9908,7 +9908,7 @@
       </c>
       <c r="K5" s="9" t="inlineStr">
         <is>
-          <t>Confirm against source report; QAS run may predate asset correction.</t>
+          <t>Source to confirm the final figure; the Quality run may predate the asset correction.</t>
         </is>
       </c>
     </row>
@@ -9959,7 +9959,7 @@
       </c>
       <c r="K6" s="9" t="inlineStr">
         <is>
-          <t>Confirm against source report; QAS run may predate asset correction.</t>
+          <t>Source to confirm the final figure; the Quality run may predate the asset correction.</t>
         </is>
       </c>
     </row>
@@ -10010,7 +10010,7 @@
       </c>
       <c r="K7" s="9" t="inlineStr">
         <is>
-          <t>Confirm against source report; QAS run may predate asset correction.</t>
+          <t>Source to confirm the final figure; the Quality run may predate the asset correction.</t>
         </is>
       </c>
     </row>
@@ -10056,12 +10056,12 @@
       </c>
       <c r="J8" s="9" t="inlineStr">
         <is>
-          <t>PRD 17,301.565 vs QAS 611.000. PRD/QAS = 28.3168: QAS carries MCF but class labels it M3.</t>
+          <t>PRD 17,301.565 vs QAS 611.000. PRD/QAS = 28.3168: Quality value is in MCF but labelled M3.</t>
         </is>
       </c>
       <c r="K8" s="9" t="inlineStr">
         <is>
-          <t>CPI to send m3 (x28.3168); fix source column for this measure.</t>
+          <t>Source to send gas in m3 (file holds MCF; multiply by 28.3168).</t>
         </is>
       </c>
     </row>
@@ -10107,12 +10107,12 @@
       </c>
       <c r="J9" s="9" t="inlineStr">
         <is>
-          <t>PRD 2,973,886.970 vs QAS 105,022.000. PRD/QAS = 28.3168: QAS carries MCF but class labels it M3.</t>
+          <t>PRD 2,973,886.970 vs QAS 105,022.000. PRD/QAS = 28.3168: Quality value is in MCF but labelled M3.</t>
         </is>
       </c>
       <c r="K9" s="9" t="inlineStr">
         <is>
-          <t>CPI to send m3 (x28.3168); fix source column for this measure.</t>
+          <t>Source to send gas in m3 (file holds MCF; multiply by 28.3168).</t>
         </is>
       </c>
     </row>
@@ -10158,12 +10158,12 @@
       </c>
       <c r="J10" s="9" t="inlineStr">
         <is>
-          <t>PRD 199,378.589 vs QAS 7,041.000. PRD/QAS = 28.3168: QAS carries MCF but class labels it M3.</t>
+          <t>PRD 199,378.589 vs QAS 7,041.000. PRD/QAS = 28.3168: Quality value is in MCF but labelled M3.</t>
         </is>
       </c>
       <c r="K10" s="9" t="inlineStr">
         <is>
-          <t>CPI to send m3 (x28.3168); fix source column for this measure.</t>
+          <t>Source to send gas in m3 (file holds MCF; multiply by 28.3168).</t>
         </is>
       </c>
     </row>
@@ -10209,12 +10209,12 @@
       </c>
       <c r="J11" s="9" t="inlineStr">
         <is>
-          <t>PRD 134,703.018 vs QAS 4,757.000. PRD/QAS = 28.3168: QAS carries MCF but class labels it M3.</t>
+          <t>PRD 134,703.018 vs QAS 4,757.000. PRD/QAS = 28.3168: Quality value is in MCF but labelled M3.</t>
         </is>
       </c>
       <c r="K11" s="9" t="inlineStr">
         <is>
-          <t>CPI to send m3 (x28.3168); fix source column for this measure.</t>
+          <t>Source to send gas in m3 (file holds MCF; multiply by 28.3168).</t>
         </is>
       </c>
     </row>
@@ -10260,12 +10260,12 @@
       </c>
       <c r="J12" s="9" t="inlineStr">
         <is>
-          <t>PRD 10,026,412.544 vs QAS 354,080.000. PRD/QAS = 28.3168: QAS carries MCF but class labels it M3.</t>
+          <t>PRD 10,026,412.544 vs QAS 354,080.000. PRD/QAS = 28.3168: Quality value is in MCF but labelled M3.</t>
         </is>
       </c>
       <c r="K12" s="9" t="inlineStr">
         <is>
-          <t>CPI to send m3 (x28.3168); fix source column for this measure.</t>
+          <t>Source to send gas in m3 (file holds MCF; multiply by 28.3168).</t>
         </is>
       </c>
     </row>
@@ -10311,12 +10311,12 @@
       </c>
       <c r="J13" s="9" t="inlineStr">
         <is>
-          <t>PRD 16,527,694.973 vs QAS 583,671.000. PRD/QAS = 28.3168: QAS carries MCF but class labels it M3.</t>
+          <t>PRD 16,527,694.973 vs QAS 583,671.000. PRD/QAS = 28.3168: Quality value is in MCF but labelled M3.</t>
         </is>
       </c>
       <c r="K13" s="9" t="inlineStr">
         <is>
-          <t>CPI to send m3 (x28.3168); fix source column for this measure.</t>
+          <t>Source to send gas in m3 (file holds MCF; multiply by 28.3168).</t>
         </is>
       </c>
     </row>
@@ -10362,12 +10362,12 @@
       </c>
       <c r="J14" s="9" t="inlineStr">
         <is>
-          <t>PRD 904,240.374 vs QAS 31,933.000. PRD/QAS = 28.3168: QAS carries MCF but class labels it M3.</t>
+          <t>PRD 904,240.374 vs QAS 31,933.000. PRD/QAS = 28.3168: Quality value is in MCF but labelled M3.</t>
         </is>
       </c>
       <c r="K14" s="9" t="inlineStr">
         <is>
-          <t>CPI to send m3 (x28.3168); fix source column for this measure.</t>
+          <t>Source to send gas in m3 (file holds MCF; multiply by 28.3168).</t>
         </is>
       </c>
     </row>
@@ -10413,12 +10413,12 @@
       </c>
       <c r="J15" s="9" t="inlineStr">
         <is>
-          <t>PRD 2,435.245 vs QAS 86.000. PRD/QAS = 28.3168: QAS carries MCF but class labels it M3.</t>
+          <t>PRD 2,435.245 vs QAS 86.000. PRD/QAS = 28.3168: Quality value is in MCF but labelled M3.</t>
         </is>
       </c>
       <c r="K15" s="9" t="inlineStr">
         <is>
-          <t>CPI to send m3 (x28.3168); fix source column for this measure.</t>
+          <t>Source to send gas in m3 (file holds MCF; multiply by 28.3168).</t>
         </is>
       </c>
     </row>
@@ -10464,12 +10464,12 @@
       </c>
       <c r="J16" s="9" t="inlineStr">
         <is>
-          <t>PRD 210,592.042 vs QAS 7,437.000. PRD/QAS = 28.3168: QAS carries MCF but class labels it M3.</t>
+          <t>PRD 210,592.042 vs QAS 7,437.000. PRD/QAS = 28.3168: Quality value is in MCF but labelled M3.</t>
         </is>
       </c>
       <c r="K16" s="9" t="inlineStr">
         <is>
-          <t>CPI to send m3 (x28.3168); fix source column for this measure.</t>
+          <t>Source to send gas in m3 (file holds MCF; multiply by 28.3168).</t>
         </is>
       </c>
     </row>
@@ -10520,7 +10520,7 @@
       </c>
       <c r="K17" s="9" t="inlineStr">
         <is>
-          <t>CPI to send m3 (x28.3168); fix source column for this measure.</t>
+          <t>Source to send gas in m3 (file holds MCF; multiply by 28.3168).</t>
         </is>
       </c>
     </row>
@@ -10566,12 +10566,12 @@
       </c>
       <c r="J18" s="9" t="inlineStr">
         <is>
-          <t>PRD 73,793.581 vs QAS 2,606.000. PRD/QAS = 28.3168: QAS carries MCF but class labels it M3.</t>
+          <t>PRD 73,793.581 vs QAS 2,606.000. PRD/QAS = 28.3168: Quality value is in MCF but labelled M3.</t>
         </is>
       </c>
       <c r="K18" s="9" t="inlineStr">
         <is>
-          <t>CPI to send m3 (x28.3168); fix source column for this measure.</t>
+          <t>Source to send gas in m3 (file holds MCF; multiply by 28.3168).</t>
         </is>
       </c>
     </row>
@@ -10617,12 +10617,12 @@
       </c>
       <c r="J19" s="9" t="inlineStr">
         <is>
-          <t>PRD 5,955,192.941 vs QAS 210,306.000. PRD/QAS = 28.3168: QAS carries MCF but class labels it M3.</t>
+          <t>PRD 5,955,192.941 vs QAS 210,306.000. PRD/QAS = 28.3168: Quality value is in MCF but labelled M3.</t>
         </is>
       </c>
       <c r="K19" s="9" t="inlineStr">
         <is>
-          <t>CPI to send m3 (x28.3168); fix source column for this measure.</t>
+          <t>Source to send gas in m3 (file holds MCF; multiply by 28.3168).</t>
         </is>
       </c>
     </row>
@@ -10668,12 +10668,12 @@
       </c>
       <c r="J20" s="9" t="inlineStr">
         <is>
-          <t>PRD 6,349,929.133 vs QAS 224,246.000. PRD/QAS = 28.3168: QAS carries MCF but class labels it M3.</t>
+          <t>PRD 6,349,929.133 vs QAS 224,246.000. PRD/QAS = 28.3168: Quality value is in MCF but labelled M3.</t>
         </is>
       </c>
       <c r="K20" s="9" t="inlineStr">
         <is>
-          <t>CPI to send m3 (x28.3168); fix source column for this measure.</t>
+          <t>Source to send gas in m3 (file holds MCF; multiply by 28.3168).</t>
         </is>
       </c>
     </row>
@@ -10719,12 +10719,12 @@
       </c>
       <c r="J21" s="9" t="inlineStr">
         <is>
-          <t>PRD 447,575.341 vs QAS 15,806.000. PRD/QAS = 28.3168: QAS carries MCF but class labels it M3.</t>
+          <t>PRD 447,575.341 vs QAS 15,806.000. PRD/QAS = 28.3168: Quality value is in MCF but labelled M3.</t>
         </is>
       </c>
       <c r="K21" s="9" t="inlineStr">
         <is>
-          <t>CPI to send m3 (x28.3168); fix source column for this measure.</t>
+          <t>Source to send gas in m3 (file holds MCF; multiply by 28.3168).</t>
         </is>
       </c>
     </row>
@@ -10773,7 +10773,7 @@
       </c>
       <c r="K22" s="9" t="inlineStr">
         <is>
-          <t>Check CPI payload / mapping for this measure.</t>
+          <t>Source to include this measure in the file.</t>
         </is>
       </c>
     </row>
@@ -10822,7 +10822,7 @@
       </c>
       <c r="K23" s="9" t="inlineStr">
         <is>
-          <t>Check CPI payload / mapping for this measure.</t>
+          <t>Source to include this measure in the file.</t>
         </is>
       </c>
     </row>
@@ -10871,7 +10871,7 @@
       </c>
       <c r="K24" s="9" t="inlineStr">
         <is>
-          <t>Check CPI payload / mapping for this measure.</t>
+          <t>Source to include this measure in the file.</t>
         </is>
       </c>
     </row>
@@ -10920,7 +10920,7 @@
       </c>
       <c r="K25" s="9" t="inlineStr">
         <is>
-          <t>Check CPI payload / mapping for this measure.</t>
+          <t>Source to include this measure in the file.</t>
         </is>
       </c>
     </row>
@@ -10971,7 +10971,7 @@
       </c>
       <c r="K26" s="10" t="inlineStr">
         <is>
-          <t>Map block in CPI.</t>
+          <t>Source to send the block code SAP uses.</t>
         </is>
       </c>
     </row>
@@ -11022,7 +11022,7 @@
       </c>
       <c r="K27" s="10" t="inlineStr">
         <is>
-          <t>Map block in CPI.</t>
+          <t>Source to send the block code SAP uses.</t>
         </is>
       </c>
     </row>
@@ -11073,7 +11073,7 @@
       </c>
       <c r="K28" s="10" t="inlineStr">
         <is>
-          <t>Map block in CPI.</t>
+          <t>Source to send the block code SAP uses.</t>
         </is>
       </c>
     </row>
@@ -11124,7 +11124,7 @@
       </c>
       <c r="K29" s="10" t="inlineStr">
         <is>
-          <t>Fix COMMENT mapping in CPI (remark column).</t>
+          <t>Source to put the operator remark in the comment field only.</t>
         </is>
       </c>
     </row>
@@ -11175,7 +11175,7 @@
       </c>
       <c r="K30" s="10" t="inlineStr">
         <is>
-          <t>Map block in CPI.</t>
+          <t>Source to send the block code SAP uses.</t>
         </is>
       </c>
     </row>
@@ -11226,7 +11226,7 @@
       </c>
       <c r="K31" s="10" t="inlineStr">
         <is>
-          <t>Fix COMMENT mapping in CPI (remark column).</t>
+          <t>Source to put the operator remark in the comment field only.</t>
         </is>
       </c>
     </row>
@@ -11424,7 +11424,7 @@
       </c>
       <c r="K35" s="11" t="inlineStr">
         <is>
-          <t>Fix COMMENT mapping in CPI (remark column).</t>
+          <t>Source to put the operator remark in the comment field only.</t>
         </is>
       </c>
     </row>
@@ -11475,7 +11475,7 @@
       </c>
       <c r="K36" s="11" t="inlineStr">
         <is>
-          <t>Fix COMMENT mapping in CPI (remark column).</t>
+          <t>Source to put the operator remark in the comment field only.</t>
         </is>
       </c>
     </row>
@@ -13339,7 +13339,7 @@
       </c>
       <c r="K74" s="11" t="inlineStr">
         <is>
-          <t>Fix COMMENT mapping in CPI (remark column).</t>
+          <t>Source to put the operator remark in the comment field only.</t>
         </is>
       </c>
     </row>
@@ -13439,7 +13439,7 @@
       </c>
       <c r="K76" s="11" t="inlineStr">
         <is>
-          <t>Fix COMMENT mapping in CPI (remark column).</t>
+          <t>Source to put the operator remark in the comment field only.</t>
         </is>
       </c>
     </row>
@@ -13735,7 +13735,7 @@
       </c>
       <c r="K82" s="11" t="inlineStr">
         <is>
-          <t>Fix COMMENT mapping in CPI (remark column).</t>
+          <t>Source to put the operator remark in the comment field only.</t>
         </is>
       </c>
     </row>
@@ -13835,7 +13835,7 @@
       </c>
       <c r="K84" s="11" t="inlineStr">
         <is>
-          <t>Fix COMMENT mapping in CPI (remark column).</t>
+          <t>Source to put the operator remark in the comment field only.</t>
         </is>
       </c>
     </row>
@@ -13886,7 +13886,7 @@
       </c>
       <c r="K85" s="11" t="inlineStr">
         <is>
-          <t>Fix COMMENT mapping in CPI (remark column).</t>
+          <t>Source to put the operator remark in the comment field only.</t>
         </is>
       </c>
     </row>
@@ -14280,7 +14280,7 @@
       </c>
       <c r="K93" s="11" t="inlineStr">
         <is>
-          <t>Fix COMMENT mapping in CPI (remark column).</t>
+          <t>Source to put the operator remark in the comment field only.</t>
         </is>
       </c>
     </row>
@@ -14478,7 +14478,7 @@
       </c>
       <c r="K97" s="11" t="inlineStr">
         <is>
-          <t>Fix COMMENT mapping in CPI (remark column).</t>
+          <t>Source to put the operator remark in the comment field only.</t>
         </is>
       </c>
     </row>
@@ -14725,7 +14725,7 @@
       </c>
       <c r="K102" s="11" t="inlineStr">
         <is>
-          <t>Fix COMMENT mapping in CPI (remark column).</t>
+          <t>Source to put the operator remark in the comment field only.</t>
         </is>
       </c>
     </row>
@@ -14825,7 +14825,7 @@
       </c>
       <c r="K104" s="11" t="inlineStr">
         <is>
-          <t>Fix COMMENT mapping in CPI (remark column).</t>
+          <t>Source to put the operator remark in the comment field only.</t>
         </is>
       </c>
     </row>
@@ -14876,7 +14876,7 @@
       </c>
       <c r="K105" s="11" t="inlineStr">
         <is>
-          <t>Fix COMMENT mapping in CPI (remark column).</t>
+          <t>Source to put the operator remark in the comment field only.</t>
         </is>
       </c>
     </row>
@@ -14927,7 +14927,7 @@
       </c>
       <c r="K106" s="11" t="inlineStr">
         <is>
-          <t>Fix COMMENT mapping in CPI (remark column).</t>
+          <t>Source to put the operator remark in the comment field only.</t>
         </is>
       </c>
     </row>
@@ -14978,7 +14978,7 @@
       </c>
       <c r="K107" s="11" t="inlineStr">
         <is>
-          <t>Fix COMMENT mapping in CPI (remark column).</t>
+          <t>Source to put the operator remark in the comment field only.</t>
         </is>
       </c>
     </row>
@@ -15029,7 +15029,7 @@
       </c>
       <c r="K108" s="11" t="inlineStr">
         <is>
-          <t>Fix COMMENT mapping in CPI (remark column).</t>
+          <t>Source to put the operator remark in the comment field only.</t>
         </is>
       </c>
     </row>
@@ -15080,7 +15080,7 @@
       </c>
       <c r="K109" s="11" t="inlineStr">
         <is>
-          <t>Fix COMMENT mapping in CPI (remark column).</t>
+          <t>Source to put the operator remark in the comment field only.</t>
         </is>
       </c>
     </row>
@@ -15131,7 +15131,7 @@
       </c>
       <c r="K110" s="11" t="inlineStr">
         <is>
-          <t>Fix COMMENT mapping in CPI (remark column).</t>
+          <t>Source to put the operator remark in the comment field only.</t>
         </is>
       </c>
     </row>
@@ -15182,7 +15182,7 @@
       </c>
       <c r="K111" s="11" t="inlineStr">
         <is>
-          <t>Fix COMMENT mapping in CPI (remark column).</t>
+          <t>Source to put the operator remark in the comment field only.</t>
         </is>
       </c>
     </row>
@@ -15233,7 +15233,7 @@
       </c>
       <c r="K112" s="11" t="inlineStr">
         <is>
-          <t>Fix COMMENT mapping in CPI (remark column).</t>
+          <t>Source to put the operator remark in the comment field only.</t>
         </is>
       </c>
     </row>
@@ -15333,7 +15333,7 @@
       </c>
       <c r="K114" s="11" t="inlineStr">
         <is>
-          <t>Fix COMMENT mapping in CPI (remark column).</t>
+          <t>Source to put the operator remark in the comment field only.</t>
         </is>
       </c>
     </row>
@@ -15433,7 +15433,7 @@
       </c>
       <c r="K116" s="11" t="inlineStr">
         <is>
-          <t>Fix COMMENT mapping in CPI (remark column).</t>
+          <t>Source to put the operator remark in the comment field only.</t>
         </is>
       </c>
     </row>
@@ -15484,7 +15484,7 @@
       </c>
       <c r="K117" s="11" t="inlineStr">
         <is>
-          <t>Fix COMMENT mapping in CPI (remark column).</t>
+          <t>Source to put the operator remark in the comment field only.</t>
         </is>
       </c>
     </row>
@@ -15535,7 +15535,7 @@
       </c>
       <c r="K118" s="11" t="inlineStr">
         <is>
-          <t>Fix COMMENT mapping in CPI (remark column).</t>
+          <t>Source to put the operator remark in the comment field only.</t>
         </is>
       </c>
     </row>
@@ -15635,7 +15635,7 @@
       </c>
       <c r="K120" s="11" t="inlineStr">
         <is>
-          <t>Fix COMMENT mapping in CPI (remark column).</t>
+          <t>Source to put the operator remark in the comment field only.</t>
         </is>
       </c>
     </row>
@@ -15686,7 +15686,7 @@
       </c>
       <c r="K121" s="11" t="inlineStr">
         <is>
-          <t>Fix COMMENT mapping in CPI (remark column).</t>
+          <t>Source to put the operator remark in the comment field only.</t>
         </is>
       </c>
     </row>
@@ -15737,7 +15737,7 @@
       </c>
       <c r="K122" s="11" t="inlineStr">
         <is>
-          <t>Fix COMMENT mapping in CPI (remark column).</t>
+          <t>Source to put the operator remark in the comment field only.</t>
         </is>
       </c>
     </row>
@@ -15788,7 +15788,7 @@
       </c>
       <c r="K123" s="11" t="inlineStr">
         <is>
-          <t>Fix COMMENT mapping in CPI (remark column).</t>
+          <t>Source to put the operator remark in the comment field only.</t>
         </is>
       </c>
     </row>
@@ -15839,7 +15839,7 @@
       </c>
       <c r="K124" s="11" t="inlineStr">
         <is>
-          <t>Fix COMMENT mapping in CPI (remark column).</t>
+          <t>Source to put the operator remark in the comment field only.</t>
         </is>
       </c>
     </row>
@@ -15890,7 +15890,7 @@
       </c>
       <c r="K125" s="11" t="inlineStr">
         <is>
-          <t>Fix COMMENT mapping in CPI (remark column).</t>
+          <t>Source to put the operator remark in the comment field only.</t>
         </is>
       </c>
     </row>
@@ -15990,7 +15990,7 @@
       </c>
       <c r="K127" s="11" t="inlineStr">
         <is>
-          <t>Fix COMMENT mapping in CPI (remark column).</t>
+          <t>Source to put the operator remark in the comment field only.</t>
         </is>
       </c>
     </row>

</xml_diff>